<commit_message>
[Add] ItemParts & Image
</commit_message>
<xml_diff>
--- a/ExcelToJsonWizard-main/excel_files/ItemTable.xlsx
+++ b/ExcelToJsonWizard-main/excel_files/ItemTable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityProjectKeubung\GitHub\Invisiphobia_NullPath\ExcelToJsonWizard\excel_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityProjectKeubung\GitHub\Invisiphobia_NullPath\ExcelToJsonWizard-main\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4093C9E-5123-46E0-82FB-076DAD08135C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDABB46B-955F-4942-940F-A9E147548B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13170" yWindow="1755" windowWidth="15330" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5745" yWindow="2700" windowWidth="14325" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="40">
   <si>
     <t>key</t>
   </si>
@@ -147,10 +147,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Bookshelf</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Tablet</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -163,6 +159,26 @@
   </si>
   <si>
     <t>OneHanded</t>
+  </si>
+  <si>
+    <t>Board</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Drum can</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>s</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Box</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>None</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -502,7 +518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
@@ -724,7 +740,7 @@
         <v>1007</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C10" s="2">
         <v>10071</v>
@@ -744,62 +760,62 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>1101</v>
+        <v>1008</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C11" s="2">
-        <v>11001</v>
+        <v>10081</v>
       </c>
       <c r="D11" s="2">
-        <v>11012</v>
+        <v>10082</v>
       </c>
       <c r="E11" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F11" s="2">
         <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
-        <v>1102</v>
-      </c>
-      <c r="B12" t="s">
-        <v>34</v>
+        <v>1009</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C12" s="2">
-        <v>11031</v>
+        <v>10091</v>
       </c>
       <c r="D12" s="2">
-        <v>11032</v>
+        <v>10092</v>
       </c>
       <c r="E12" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="F12" s="2">
         <v>0</v>
       </c>
       <c r="G12" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
-        <v>1201</v>
+        <v>1101</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C13" s="2">
-        <v>11021</v>
+        <v>11001</v>
       </c>
       <c r="D13" s="2">
-        <v>11022</v>
+        <v>11012</v>
       </c>
       <c r="E13" t="s">
         <v>14</v>
@@ -808,6 +824,52 @@
         <v>0</v>
       </c>
       <c r="G13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
+        <v>1102</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="2">
+        <v>11031</v>
+      </c>
+      <c r="D14" s="2">
+        <v>11032</v>
+      </c>
+      <c r="E14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
+      </c>
+      <c r="G14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
+        <v>1201</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="2">
+        <v>11021</v>
+      </c>
+      <c r="D15" s="2">
+        <v>11022</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
+      <c r="G15" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[Update] Door & lock
문과 자물쇠 상호작용 액셀 내용 추가 및
스크립트에 적용.
</commit_message>
<xml_diff>
--- a/ExcelToJsonWizard-main/excel_files/ItemTable.xlsx
+++ b/ExcelToJsonWizard-main/excel_files/ItemTable.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="2670" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="3600" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -931,7 +931,7 @@
         <v>10081</v>
       </c>
       <c r="D11" s="2">
-        <v>-1</v>
+        <v>10082</v>
       </c>
       <c r="E11" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
[Update] Lock, Tablet item, Hacking
아이템 얻거나 상호작용 시 나올 대사 삽입 및 버그 수정.
</commit_message>
<xml_diff>
--- a/ExcelToJsonWizard-main/excel_files/ItemTable.xlsx
+++ b/ExcelToJsonWizard-main/excel_files/ItemTable.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="3600" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="4530" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="62">
   <si>
     <t>key</t>
   </si>
@@ -259,6 +259,10 @@
   </si>
   <si>
     <t>에러메시지</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>10102,10103</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -988,8 +992,8 @@
       <c r="C13" s="2">
         <v>10101</v>
       </c>
-      <c r="D13" s="2">
-        <v>-1</v>
+      <c r="D13" s="7" t="s">
+        <v>61</v>
       </c>
       <c r="E13" t="s">
         <v>12</v>

</xml_diff>